<commit_message>
Module 1: reframe mean/median subsection around the mean-median gap and outliers; demote skew to a vocabulary note
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0165WQeoaB3CPsnpvD7o3Yah
</commit_message>
<xml_diff>
--- a/barley_varieties_2025_rz1.xlsx
+++ b/barley_varieties_2025_rz1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usaskca1-my.sharepoint.com/personal/pjs998_usask_ca/Documents/Teaching/261/2026/textbook_261/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="81" documentId="8_{90BDDC2B-06A7-3E4B-9CEF-08BC670C7BB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EA64C25B-226C-0D4E-A94C-C66047F01016}"/>
+  <xr:revisionPtr revIDLastSave="82" documentId="8_{90BDDC2B-06A7-3E4B-9CEF-08BC670C7BB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{64DE6167-F5F4-4743-9C15-35C02EDF60FE}"/>
   <bookViews>
-    <workbookView xWindow="5580" yWindow="2380" windowWidth="27640" windowHeight="16680" xr2:uid="{CEFF5260-15F5-3341-8604-A454612919C2}"/>
+    <workbookView xWindow="4960" yWindow="1780" windowWidth="27640" windowHeight="16680" xr2:uid="{CEFF5260-15F5-3341-8604-A454612919C2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -675,6 +675,10 @@
       <c r="A11" t="s">
         <v>15</v>
       </c>
+      <c r="C11">
+        <f>AVERAGE(C2:C10)</f>
+        <v>90.811111111111103</v>
+      </c>
       <c r="D11">
         <f>D2+D3+D4+D5+D6+D7+D8+D9+D10</f>
         <v>2886795.4</v>

</xml_diff>

<commit_message>
Module 1: add Weighted Average subsection after Mean (barley acreage-weighted example + course-grade example)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0165WQeoaB3CPsnpvD7o3Yah
</commit_message>
<xml_diff>
--- a/barley_varieties_2025_rz1.xlsx
+++ b/barley_varieties_2025_rz1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usaskca1-my.sharepoint.com/personal/pjs998_usask_ca/Documents/Teaching/261/2026/textbook_261/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="82" documentId="8_{90BDDC2B-06A7-3E4B-9CEF-08BC670C7BB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{64DE6167-F5F4-4743-9C15-35C02EDF60FE}"/>
+  <xr:revisionPtr revIDLastSave="86" documentId="8_{90BDDC2B-06A7-3E4B-9CEF-08BC670C7BB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0E370454-E3D5-0645-8562-F419C91DD9E3}"/>
   <bookViews>
     <workbookView xWindow="4960" yWindow="1780" windowWidth="27640" windowHeight="16680" xr2:uid="{CEFF5260-15F5-3341-8604-A454612919C2}"/>
   </bookViews>
@@ -675,16 +675,16 @@
       <c r="A11" t="s">
         <v>15</v>
       </c>
-      <c r="C11">
-        <f>AVERAGE(C2:C10)</f>
-        <v>90.811111111111103</v>
-      </c>
       <c r="D11">
         <f>D2+D3+D4+D5+D6+D7+D8+D9+D10</f>
         <v>2886795.4</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B12">
+        <f>AVERAGE(B2:B10)</f>
+        <v>3503.3333333333335</v>
+      </c>
       <c r="D12">
         <f>SUM(D2:D10)</f>
         <v>2886795.4</v>
@@ -695,6 +695,10 @@
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B13">
+        <f>MEDIAN(B2:B10)</f>
+        <v>2029</v>
+      </c>
       <c r="D13">
         <f>SUM(Production)</f>
         <v>2886795.4</v>

</xml_diff>

<commit_message>
Module 1: integrate cell formatting into The Basics (value vs display, displayed-rounding gotcha)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0165WQeoaB3CPsnpvD7o3Yah
</commit_message>
<xml_diff>
--- a/barley_varieties_2025_rz1.xlsx
+++ b/barley_varieties_2025_rz1.xlsx
@@ -8,16 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usaskca1-my.sharepoint.com/personal/pjs998_usask_ca/Documents/Teaching/261/2026/textbook_261/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="86" documentId="8_{90BDDC2B-06A7-3E4B-9CEF-08BC670C7BB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0E370454-E3D5-0645-8562-F419C91DD9E3}"/>
+  <xr:revisionPtr revIDLastSave="167" documentId="8_{90BDDC2B-06A7-3E4B-9CEF-08BC670C7BB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FB8A8782-7C46-9D44-A746-FE3D89140C5D}"/>
   <bookViews>
-    <workbookView xWindow="4960" yWindow="1780" windowWidth="27640" windowHeight="16680" xr2:uid="{CEFF5260-15F5-3341-8604-A454612919C2}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="25800" windowHeight="20460" xr2:uid="{CEFF5260-15F5-3341-8604-A454612919C2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="price">Sheet1!$B$14</definedName>
-    <definedName name="Production">Sheet1!$D$2:$D$10</definedName>
+    <definedName name="price">Sheet1!#REF!</definedName>
+    <definedName name="Production">Sheet1!#REF!</definedName>
+    <definedName name="Production2">Sheet1!$D$2:$D$10</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>Variety</t>
   </si>
@@ -81,23 +82,32 @@
     <t>Yield (bu/ac)</t>
   </si>
   <si>
-    <t>Production</t>
-  </si>
-  <si>
-    <t>Revenue</t>
-  </si>
-  <si>
     <t>Barley price</t>
   </si>
   <si>
-    <t>Total production</t>
+    <t>Total production (bu)</t>
+  </si>
+  <si>
+    <t>Revenue ($)</t>
+  </si>
+  <si>
+    <t>Totals</t>
+  </si>
+  <si>
+    <t>Average</t>
+  </si>
+  <si>
+    <t>Weighted average</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+  </numFmts>
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -105,8 +115,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -116,12 +133,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -138,10 +149,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -476,11 +488,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BB414AF-48AF-3748-9D71-C9332721118C}">
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="17.33203125" customWidth="1"/>
+    <col min="5" max="5" width="15.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
@@ -494,10 +508,10 @@
         <v>11</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
@@ -514,8 +528,8 @@
         <f>B2*C2</f>
         <v>60216</v>
       </c>
-      <c r="E2">
-        <f>D2*price</f>
+      <c r="E2" s="2">
+        <f>D2*$B$17</f>
         <v>331188</v>
       </c>
     </row>
@@ -533,8 +547,8 @@
         <f t="shared" ref="D3:D10" si="0">B3*C3</f>
         <v>279122.80000000005</v>
       </c>
-      <c r="E3">
-        <f>D3*price</f>
+      <c r="E3" s="2">
+        <f t="shared" ref="E3:E11" si="1">D3*$B$17</f>
         <v>1535175.4000000004</v>
       </c>
     </row>
@@ -552,8 +566,8 @@
         <f t="shared" si="0"/>
         <v>194805</v>
       </c>
-      <c r="E4">
-        <f>D4*price</f>
+      <c r="E4" s="2">
+        <f t="shared" si="1"/>
         <v>1071427.5</v>
       </c>
     </row>
@@ -571,8 +585,8 @@
         <f t="shared" si="0"/>
         <v>207972.5</v>
       </c>
-      <c r="E5">
-        <f>D5*price</f>
+      <c r="E5" s="2">
+        <f t="shared" si="1"/>
         <v>1143848.75</v>
       </c>
     </row>
@@ -587,11 +601,11 @@
         <v>87.5</v>
       </c>
       <c r="D6">
-        <f t="shared" si="0"/>
+        <f>B6*C6</f>
         <v>350350</v>
       </c>
-      <c r="E6">
-        <f>D6*price</f>
+      <c r="E6" s="2">
+        <f t="shared" si="1"/>
         <v>1926925</v>
       </c>
     </row>
@@ -606,11 +620,11 @@
         <v>95.9</v>
       </c>
       <c r="D7">
-        <f t="shared" si="0"/>
+        <f>B7*C7</f>
         <v>752815</v>
       </c>
-      <c r="E7">
-        <f>D7*price</f>
+      <c r="E7" s="2">
+        <f t="shared" si="1"/>
         <v>4140482.5</v>
       </c>
     </row>
@@ -628,8 +642,8 @@
         <f t="shared" si="0"/>
         <v>109318.39999999999</v>
       </c>
-      <c r="E8">
-        <f>D8*price</f>
+      <c r="E8" s="2">
+        <f t="shared" si="1"/>
         <v>601251.19999999995</v>
       </c>
     </row>
@@ -647,8 +661,8 @@
         <f t="shared" si="0"/>
         <v>108644.40000000001</v>
       </c>
-      <c r="E9">
-        <f>D9*price</f>
+      <c r="E9" s="2">
+        <f t="shared" si="1"/>
         <v>597544.20000000007</v>
       </c>
     </row>
@@ -666,53 +680,56 @@
         <f t="shared" si="0"/>
         <v>823551.29999999993</v>
       </c>
-      <c r="E10">
-        <f>D10*price</f>
+      <c r="E10" s="2">
+        <f t="shared" si="1"/>
         <v>4529532.1499999994</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
+      <c r="A11" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D11">
+      <c r="B11" s="3">
+        <f>SUM(B2:B10)</f>
+        <v>31530</v>
+      </c>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3">
         <f>D2+D3+D4+D5+D6+D7+D8+D9+D10</f>
         <v>2886795.4</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B12">
-        <f>AVERAGE(B2:B10)</f>
+      <c r="E11" s="2">
+        <f t="shared" si="1"/>
+        <v>15877374.699999999</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13">
+        <f>SUM(B2:B10)/9</f>
         <v>3503.3333333333335</v>
       </c>
-      <c r="D12">
-        <f>SUM(D2:D10)</f>
-        <v>2886795.4</v>
-      </c>
-      <c r="E12">
-        <f>SUM(E2:E10)</f>
-        <v>15877374.699999999</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B13">
-        <f>MEDIAN(B2:B10)</f>
-        <v>2029</v>
-      </c>
-      <c r="D13">
-        <f>SUM(Production)</f>
-        <v>2886795.4</v>
-      </c>
-      <c r="E13">
-        <f>SUM(Production)</f>
-        <v>2886795.4</v>
+      <c r="C13">
+        <f>AVERAGE(C2:C10)</f>
+        <v>90.811111111111103</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A14" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B14" s="2">
+      <c r="A14" t="s">
+        <v>17</v>
+      </c>
+      <c r="C14">
+        <f>D11/B11</f>
+        <v>91.557101173485563</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>12</v>
+      </c>
+      <c r="B17" s="2">
         <v>5.5</v>
       </c>
     </row>

</xml_diff>